<commit_message>
feat(reporter): custom report improvements
</commit_message>
<xml_diff>
--- a/data/ui/testRegistry.xlsx
+++ b/data/ui/testRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manishgangwar/LearnPlaywright/data/ui/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{404CCBA2-9C9D-0D44-9514-88A6E9FB7475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4AA312A-69F1-D44A-B1B5-A7649D9E20C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10360" yWindow="1780" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{20BDFCB9-813F-5B44-AE4E-B81527177D88}"/>
   </bookViews>
@@ -731,7 +731,7 @@
         <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -889,7 +889,7 @@
         <v>35</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -900,7 +900,7 @@
         <v>37</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>